<commit_message>
Book bonus provision (8.33% on Basic+DA, eligible <=21k/mo) into restated Maharashtra financials
- Note 16 Employee Benefit Expense: +Rs 20,492,342.50 bonus line -> 364,293,736
- Note 12 Other Payables and Provisions: Bonus Payable 20,492,342.50 -> total 22,171,974.50
- P&L Total Expenses 439,780,145.12; Surplus before tax 133,151,366.98
- Balance Sheet unchanged at 217,022,982.71 (surplus down, payable up)
</commit_message>
<xml_diff>
--- a/docs/maharashtra/Maharashtra_Financials_FY24-25_Restated.xlsx
+++ b/docs/maharashtra/Maharashtra_Financials_FY24-25_Restated.xlsx
@@ -523,6 +523,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -628,7 +629,7 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>343801393.5</v>
+        <v>364293736</v>
       </c>
     </row>
     <row r="13">
@@ -684,7 +685,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr"/>
       <c r="C16" s="8" t="n">
-        <v>419287802.62</v>
+        <v>439780145.12</v>
       </c>
     </row>
     <row r="17">
@@ -695,7 +696,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr"/>
       <c r="C17" s="8" t="n">
-        <v>153643709.48</v>
+        <v>133151366.98</v>
       </c>
     </row>
   </sheetData>
@@ -736,6 +737,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -913,7 +915,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr"/>
       <c r="C17" s="6" t="n">
-        <v>153643709.48</v>
+        <v>133151366.98</v>
       </c>
     </row>
     <row r="18">
@@ -958,7 +960,7 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>1679632</v>
+        <v>22171974.5</v>
       </c>
     </row>
     <row r="21">
@@ -1017,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1034,6 +1036,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -1170,6 +1173,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
@@ -1197,6 +1201,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
@@ -1224,6 +1229,7 @@
         <v>152488866.3</v>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
@@ -1251,6 +1257,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -1278,6 +1285,7 @@
         <v>4248</v>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
@@ -1325,6 +1333,7 @@
         <v>76981.74000000001</v>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
@@ -1352,6 +1361,7 @@
         <v>44704175</v>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
@@ -1456,6 +1466,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
@@ -1560,6 +1571,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
@@ -1637,6 +1649,7 @@
         <v>12149631.4</v>
       </c>
     </row>
+    <row r="70"/>
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
         <is>
@@ -1664,6 +1677,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="74"/>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
         <is>
@@ -1698,7 +1712,7 @@
         </is>
       </c>
       <c r="C78" s="13" t="n">
-        <v>0</v>
+        <v>20492342.5</v>
       </c>
     </row>
     <row r="79">
@@ -1718,9 +1732,10 @@
         </is>
       </c>
       <c r="C80" s="15" t="n">
-        <v>1679632</v>
-      </c>
-    </row>
+        <v>22171974.5</v>
+      </c>
+    </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
@@ -1778,6 +1793,7 @@
         <v>572931512.1</v>
       </c>
     </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="11" t="inlineStr">
         <is>
@@ -1885,6 +1901,7 @@
         <v>10893518.66</v>
       </c>
     </row>
+    <row r="100"/>
     <row r="101">
       <c r="A101" s="11" t="inlineStr">
         <is>
@@ -2042,6 +2059,7 @@
         <v>60263172.83</v>
       </c>
     </row>
+    <row r="117"/>
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
@@ -2130,250 +2148,263 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="14" t="inlineStr">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Bonus (provision @ 8.33% on Basic+DA, eligible &lt;= Rs.21,000/mo - Payment of Bonus Act)</t>
+        </is>
+      </c>
+      <c r="C127" s="13" t="n">
+        <v>20492342.5</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C127" s="15" t="n">
-        <v>343801393.5</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="11" t="inlineStr">
+      <c r="C128" s="15" t="n">
+        <v>364293736</v>
+      </c>
+    </row>
+    <row r="129"/>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
         <is>
           <t>Note 17 - Finance Costs</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
+    <row r="131">
+      <c r="A131" t="inlineStr">
         <is>
           <t>GST Interest</t>
         </is>
       </c>
-      <c r="C130" s="13" t="n">
+      <c r="C131" s="13" t="n">
         <v>2451</v>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="14" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="14" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C131" s="15" t="n">
+      <c r="C132" s="15" t="n">
         <v>2451</v>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="11" t="inlineStr">
+    <row r="133"/>
+    <row r="134">
+      <c r="A134" s="11" t="inlineStr">
         <is>
           <t>Note 18 - Depreciation (as per fixed-asset schedule)</t>
         </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>Depreciation - Computer</t>
-        </is>
-      </c>
-      <c r="C134" s="13" t="n">
-        <v>448320.16</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Depreciation - Office Equipment</t>
+          <t>Depreciation - Computer</t>
         </is>
       </c>
       <c r="C135" s="13" t="n">
-        <v>42045.6</v>
+        <v>448320.16</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Depreciation - Plant &amp; Machinery</t>
+          <t>Depreciation - Office Equipment</t>
         </is>
       </c>
       <c r="C136" s="13" t="n">
-        <v>1441925.23</v>
+        <v>42045.6</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>Depreciation - Plant &amp; Machinery</t>
+        </is>
+      </c>
+      <c r="C137" s="13" t="n">
+        <v>1441925.23</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
           <t>Depreciation - Building</t>
         </is>
       </c>
-      <c r="C137" s="13" t="n">
+      <c r="C138" s="13" t="n">
         <v>672136.72</v>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="14" t="inlineStr">
+    <row r="139">
+      <c r="A139" s="14" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C138" s="15" t="n">
+      <c r="C139" s="15" t="n">
         <v>2604427.71</v>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="3" t="inlineStr">
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
         <is>
           <t>(Earlier TB depreciation of Rs 47,525.42 on Computer reversed; full-year depreciation taken per schedule.)</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="11" t="inlineStr">
+    <row r="141"/>
+    <row r="142">
+      <c r="A142" s="11" t="inlineStr">
         <is>
           <t>Note 19 - Other Expenses</t>
         </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Communication Expenses</t>
-        </is>
-      </c>
-      <c r="C142" s="13" t="n">
-        <v>175825.02</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Travelling &amp; Conveyance</t>
+          <t>Communication Expenses</t>
         </is>
       </c>
       <c r="C143" s="13" t="n">
-        <v>128830.08</v>
+        <v>175825.02</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Electricity &amp; Water</t>
+          <t>Travelling &amp; Conveyance</t>
         </is>
       </c>
       <c r="C144" s="13" t="n">
-        <v>263240</v>
+        <v>128830.08</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Legal &amp; Professional Charges</t>
+          <t>Electricity &amp; Water</t>
         </is>
       </c>
       <c r="C145" s="13" t="n">
-        <v>100000</v>
+        <v>263240</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Fees &amp; Taxes</t>
+          <t>Legal &amp; Professional Charges</t>
         </is>
       </c>
       <c r="C146" s="13" t="n">
-        <v>103732</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Fooding Deduction</t>
+          <t>Fees &amp; Taxes</t>
         </is>
       </c>
       <c r="C147" s="13" t="n">
-        <v>66193</v>
+        <v>103732</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Other Deduction</t>
+          <t>Fooding Deduction</t>
         </is>
       </c>
       <c r="C148" s="13" t="n">
-        <v>12741.63</v>
+        <v>66193</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Miscellaneous Expenses (net of round off)</t>
+          <t>Other Deduction</t>
         </is>
       </c>
       <c r="C149" s="13" t="n">
-        <v>240352.19</v>
+        <v>12741.63</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Diwali Expenses</t>
+          <t>Miscellaneous Expenses (net of round off)</t>
         </is>
       </c>
       <c r="C150" s="13" t="n">
-        <v>51000</v>
+        <v>240352.19</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Printing &amp; Stationery</t>
+          <t>Diwali Expenses</t>
         </is>
       </c>
       <c r="C151" s="13" t="n">
-        <v>172599</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Repair and Maintenance - Machinery</t>
+          <t>Printing &amp; Stationery</t>
         </is>
       </c>
       <c r="C152" s="13" t="n">
-        <v>43088</v>
+        <v>172599</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Other Repairs</t>
+          <t>Repair and Maintenance - Machinery</t>
         </is>
       </c>
       <c r="C153" s="13" t="n">
-        <v>11238</v>
+        <v>43088</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
+          <t>Other Repairs</t>
+        </is>
+      </c>
+      <c r="C154" s="13" t="n">
+        <v>11238</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
           <t>Rent</t>
         </is>
       </c>
-      <c r="C154" s="13" t="n">
+      <c r="C155" s="13" t="n">
         <v>354000</v>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="14" t="inlineStr">
+    <row r="156">
+      <c r="A156" s="14" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C155" s="15" t="n">
+      <c r="C156" s="15" t="n">
         <v>1722838.92</v>
       </c>
     </row>

</xml_diff>